<commit_message>
Add Badera and Domsi-Makhdet DI site reports to the dataset
- Badeda Spring (RDI-SPR-0008) and Makhdet Spring (RDI-SPR-0009) from the SRHU
  hydrogeological assessment reports (SRC-027, SRC-028): coordinates, geology,
  spring type, surface catchment and land use. Neither report gives discharge.
- The Kunjapuri DI handpump from the field visit is the Badera report's
  handpump; it is linked to Badeda Spring (68 m above it, 189 m away on the DEM).
- Map values built for the two new records only.

1,845 records, 1,680 distinct springs (input 1,463 unchanged, test 217).

Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01SYEMBaPiJtYrK4Gc2Fn2t3
</commit_message>
<xml_diff>
--- a/data/01_staged/literature/xlsx/literature_spring_records_common_v1.xlsx
+++ b/data/01_staged/literature/xlsx/literature_spring_records_common_v1.xlsx
@@ -457,7 +457,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AW54"/>
+  <dimension ref="A1:AW56"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -7741,6 +7741,324 @@
         </is>
       </c>
     </row>
+    <row r="55">
+      <c r="A55" s="2" t="inlineStr">
+        <is>
+          <t>RDI-SPR-0008</t>
+        </is>
+      </c>
+      <c r="B55" s="2" t="inlineStr">
+        <is>
+          <t>SRC-027</t>
+        </is>
+      </c>
+      <c r="C55" s="2" t="inlineStr">
+        <is>
+          <t>RDI/WATSAN (SRHU) DI site hydrogeological assessment report</t>
+        </is>
+      </c>
+      <c r="D55" s="2" t="inlineStr">
+        <is>
+          <t>Badera Geohydrology  report.pdf, section 1 (Location and Site Characteristics)</t>
+        </is>
+      </c>
+      <c r="E55" s="2" t="inlineStr">
+        <is>
+          <t>Badeda village, Narendra Nagar block, Tehri Garhwal, Uttarakhand</t>
+        </is>
+      </c>
+      <c r="F55" s="2" t="inlineStr">
+        <is>
+          <t>Tehri Garhwal</t>
+        </is>
+      </c>
+      <c r="G55" s="2" t="inlineStr">
+        <is>
+          <t>Narendra Nagar</t>
+        </is>
+      </c>
+      <c r="H55" s="2" t="inlineStr"/>
+      <c r="I55" s="2" t="inlineStr">
+        <is>
+          <t>Badeda (Badera)</t>
+        </is>
+      </c>
+      <c r="J55" s="2" t="inlineStr">
+        <is>
+          <t>Badeda Spring</t>
+        </is>
+      </c>
+      <c r="K55" s="2" t="inlineStr">
+        <is>
+          <t>30.171461</t>
+        </is>
+      </c>
+      <c r="L55" s="2" t="inlineStr">
+        <is>
+          <t>78.312894</t>
+        </is>
+      </c>
+      <c r="M55" s="2" t="inlineStr"/>
+      <c r="N55" s="2" t="inlineStr">
+        <is>
+          <t>Catchment: dense forest 48.4 %, open forest 16.0 %, agriculture/terrace 25.7 %, built-up 5.2 %, barren 3.2 %, road 1.5 % (Sentinel-2, 2025; the text says 66.91 % forest)</t>
+        </is>
+      </c>
+      <c r="O55" s="2" t="inlineStr"/>
+      <c r="P55" s="2" t="inlineStr"/>
+      <c r="Q55" s="2" t="inlineStr">
+        <is>
+          <t>Limestone, dolomite and shale (Krol Group); aquifer table adds quartzite and sandstone (Blaini Group)</t>
+        </is>
+      </c>
+      <c r="R55" s="2" t="inlineStr">
+        <is>
+          <t>Fracture-controlled contact spring; fractured to semi-confined carbonate aquifer of the Krol Group</t>
+        </is>
+      </c>
+      <c r="S55" s="2" t="inlineStr"/>
+      <c r="T55" s="2" t="inlineStr"/>
+      <c r="U55" s="2" t="inlineStr"/>
+      <c r="V55" s="2" t="inlineStr"/>
+      <c r="W55" s="2" t="inlineStr">
+        <is>
+          <t>Perennial</t>
+        </is>
+      </c>
+      <c r="X55" s="2" t="inlineStr"/>
+      <c r="Y55" s="2" t="inlineStr">
+        <is>
+          <t>Neoproterozoic Krol Group; groundwater controlled by fractures, joints and bedding planes; Highly Dissected Structural Hills and Valleys</t>
+        </is>
+      </c>
+      <c r="Z55" s="2" t="inlineStr">
+        <is>
+          <t>Secondary porosity through fractures, joints and weathering (soil effective porosity 25-40 %)</t>
+        </is>
+      </c>
+      <c r="AA55" s="2" t="inlineStr"/>
+      <c r="AB55" s="2" t="inlineStr"/>
+      <c r="AC55" s="2" t="inlineStr">
+        <is>
+          <t>POINT (78.312894 30.171461)</t>
+        </is>
+      </c>
+      <c r="AD55" s="2" t="inlineStr">
+        <is>
+          <t>Verify: no spring discharge is reported; the catchment is a surface delineation, not a recharge area; the handpump-spring link is the report's interpretation.</t>
+        </is>
+      </c>
+      <c r="AE55" s="2" t="inlineStr">
+        <is>
+          <t>Transcribed from the report text and the land use table; coordinates converted from degrees-minutes-seconds.</t>
+        </is>
+      </c>
+      <c r="AF55" s="2" t="inlineStr">
+        <is>
+          <t>Swami Rama Himalayan University (RDI/WATSAN). Scientific Hydrogeological Assessment Report - Impact Assessment of Direct Injection-Based Aquifer Recharge Technique for Spring Revival: Badeda village, Narendra Nagar block, Tehri Garhwal, Uttarakhand (Badera Geohydrology  report.pdf, undated)</t>
+        </is>
+      </c>
+      <c r="AG55" s="2" t="inlineStr">
+        <is>
+          <t>Coordinates printed to 0.01 second; no discharge or water quality; areas are surface catchments.</t>
+        </is>
+      </c>
+      <c r="AH55" s="2" t="inlineStr">
+        <is>
+          <t>Surface catchment from CartoDEM 30 m with thematic layers; the handpump area is called the upper recharge zone</t>
+        </is>
+      </c>
+      <c r="AI55" s="2" t="inlineStr"/>
+      <c r="AJ55" s="2" t="inlineStr"/>
+      <c r="AK55" s="2" t="inlineStr"/>
+      <c r="AL55" s="2" t="inlineStr"/>
+      <c r="AM55" s="2" t="inlineStr">
+        <is>
+          <t>40.51</t>
+        </is>
+      </c>
+      <c r="AN55" s="2" t="inlineStr">
+        <is>
+          <t>1452–1614</t>
+        </is>
+      </c>
+      <c r="AO55" s="2" t="inlineStr"/>
+      <c r="AP55" s="2" t="inlineStr"/>
+      <c r="AQ55" s="2" t="inlineStr"/>
+      <c r="AR55" s="2" t="inlineStr"/>
+      <c r="AS55" s="2" t="inlineStr"/>
+      <c r="AT55" s="2" t="inlineStr">
+        <is>
+          <t>Slope 5–36° (12–28° around the handpump); mostly south- to southwest-facing</t>
+        </is>
+      </c>
+      <c r="AU55" s="2" t="inlineStr">
+        <is>
+          <t>Rooftop rainwater harvesting with direct injection through the existing Badeda handpump (Kunjapuri; report: 'upper recharge zone of the Kunjapuri Spring catchment') at 30.173392, 78.312847, plus catchment treatment (trenches, recharge pits, check dams). The report places the handpump upslope of the spring in the same shallow fractured aquifer ('only a few metres apart'; the printed coordinates are about 215 m apart).</t>
+        </is>
+      </c>
+      <c r="AV55" s="2" t="inlineStr"/>
+      <c r="AW55" s="2" t="inlineStr"/>
+    </row>
+    <row r="56">
+      <c r="A56" s="2" t="inlineStr">
+        <is>
+          <t>RDI-SPR-0009</t>
+        </is>
+      </c>
+      <c r="B56" s="2" t="inlineStr">
+        <is>
+          <t>SRC-028</t>
+        </is>
+      </c>
+      <c r="C56" s="2" t="inlineStr">
+        <is>
+          <t>RDI/WATSAN (SRHU) DI site hydrogeological assessment report</t>
+        </is>
+      </c>
+      <c r="D56" s="2" t="inlineStr">
+        <is>
+          <t>Domsi &amp; Makhdet Geohydrology report.pdf, section 1 (Location and Site Characteristics)</t>
+        </is>
+      </c>
+      <c r="E56" s="2" t="inlineStr">
+        <is>
+          <t>Dungsi &amp; Makhdet villages, Jaunpur block, Tehri Garhwal, Uttarakhand</t>
+        </is>
+      </c>
+      <c r="F56" s="2" t="inlineStr">
+        <is>
+          <t>Tehri Garhwal</t>
+        </is>
+      </c>
+      <c r="G56" s="2" t="inlineStr">
+        <is>
+          <t>Jaunpur</t>
+        </is>
+      </c>
+      <c r="H56" s="2" t="inlineStr"/>
+      <c r="I56" s="2" t="inlineStr">
+        <is>
+          <t>Makhdet (Dungsi &amp; Makhdet; also spelt Madkhet, Domsi)</t>
+        </is>
+      </c>
+      <c r="J56" s="2" t="inlineStr">
+        <is>
+          <t>Makhdet Spring</t>
+        </is>
+      </c>
+      <c r="K56" s="2" t="inlineStr">
+        <is>
+          <t>30.482739</t>
+        </is>
+      </c>
+      <c r="L56" s="2" t="inlineStr">
+        <is>
+          <t>78.234675</t>
+        </is>
+      </c>
+      <c r="M56" s="2" t="inlineStr"/>
+      <c r="N56" s="2" t="inlineStr">
+        <is>
+          <t>Catchment: dense forest 40.8 %, open forest 25.4 %, agriculture/terrace 22.6 %, built-up 4.3 %, barren 3.5 %, road 1.3 %, water 0.3 % (Sentinel-2, 2025)</t>
+        </is>
+      </c>
+      <c r="O56" s="2" t="inlineStr"/>
+      <c r="P56" s="2" t="inlineStr"/>
+      <c r="Q56" s="2" t="inlineStr">
+        <is>
+          <t>Quartzite, phyllite, slate and schist (Jaunsar Group; the aquifer table says Jaunpur Group)</t>
+        </is>
+      </c>
+      <c r="R56" s="2" t="inlineStr">
+        <is>
+          <t>Fracture-controlled gravity spring; unconfined to semi-confined fractured hard-rock aquifer</t>
+        </is>
+      </c>
+      <c r="S56" s="2" t="inlineStr"/>
+      <c r="T56" s="2" t="inlineStr"/>
+      <c r="U56" s="2" t="inlineStr"/>
+      <c r="V56" s="2" t="inlineStr"/>
+      <c r="W56" s="2" t="inlineStr">
+        <is>
+          <t>Perennial</t>
+        </is>
+      </c>
+      <c r="X56" s="2" t="inlineStr"/>
+      <c r="Y56" s="2" t="inlineStr">
+        <is>
+          <t>Neoproterozoic Jaunsar Group, Lesser Himalaya; groundwater controlled by fractures, joints, foliation and bedding planes; Highly Dissected Hills and Valleys</t>
+        </is>
+      </c>
+      <c r="Z56" s="2" t="inlineStr">
+        <is>
+          <t>Secondary porosity through fractures, joints, foliation and weathering (soil effective porosity 20-35 %)</t>
+        </is>
+      </c>
+      <c r="AA56" s="2" t="inlineStr"/>
+      <c r="AB56" s="2" t="inlineStr"/>
+      <c r="AC56" s="2" t="inlineStr">
+        <is>
+          <t>POINT (78.234675 30.482739)</t>
+        </is>
+      </c>
+      <c r="AD56" s="2" t="inlineStr">
+        <is>
+          <t>Verify: no spring discharge is reported; the catchment is a surface delineation, not a recharge area; the handpump-spring link is the report's interpretation.</t>
+        </is>
+      </c>
+      <c r="AE56" s="2" t="inlineStr">
+        <is>
+          <t>Transcribed from the report text and the land use table; coordinates converted from degrees-minutes-seconds.</t>
+        </is>
+      </c>
+      <c r="AF56" s="2" t="inlineStr">
+        <is>
+          <t>Swami Rama Himalayan University (RDI/WATSAN). Scientific Hydrogeological Assessment Report - Impact Assessment of Direct Injection-Based Aquifer Recharge Technique for Spring Revival: Dungsi &amp; Makhdet villages, Jaunpur block, Tehri Garhwal, Uttarakhand (Domsi &amp; Makhdet Geohydrology report.pdf, undated)</t>
+        </is>
+      </c>
+      <c r="AG56" s="2" t="inlineStr">
+        <is>
+          <t>Coordinates printed to 0.01 second; no discharge or water quality; areas are surface catchments.</t>
+        </is>
+      </c>
+      <c r="AH56" s="2" t="inlineStr">
+        <is>
+          <t>Surface catchment from CartoDEM 30 m with thematic layers; the handpump area is called the upper recharge zone</t>
+        </is>
+      </c>
+      <c r="AI56" s="2" t="inlineStr"/>
+      <c r="AJ56" s="2" t="inlineStr"/>
+      <c r="AK56" s="2" t="inlineStr"/>
+      <c r="AL56" s="2" t="inlineStr"/>
+      <c r="AM56" s="2" t="inlineStr">
+        <is>
+          <t>91.07</t>
+        </is>
+      </c>
+      <c r="AN56" s="2" t="inlineStr">
+        <is>
+          <t>1461–2076</t>
+        </is>
+      </c>
+      <c r="AO56" s="2" t="inlineStr"/>
+      <c r="AP56" s="2" t="inlineStr"/>
+      <c r="AQ56" s="2" t="inlineStr"/>
+      <c r="AR56" s="2" t="inlineStr"/>
+      <c r="AS56" s="2" t="inlineStr"/>
+      <c r="AT56" s="2" t="inlineStr">
+        <is>
+          <t>Slope 5 to over 37° (5–15° around the spring and handpump); spring and handpump on northwest-facing slopes</t>
+        </is>
+      </c>
+      <c r="AU56" s="2" t="inlineStr">
+        <is>
+          <t>Rooftop rainwater harvesting with direct injection through the existing Dungsi (Domsi) handpump at 30.481472, 78.236694, plus catchment treatment (trenches, recharge pits, check dams). The report places the handpump upslope of the spring in the same springshed, with 'probable hydraulic connectivity' through the fractured aquifer.</t>
+        </is>
+      </c>
+      <c r="AV56" s="2" t="inlineStr"/>
+      <c r="AW56" s="2" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -7785,7 +8103,7 @@
         </is>
       </c>
       <c r="B3" s="5" t="n">
-        <v>53</v>
+        <v>55</v>
       </c>
     </row>
     <row r="4">
@@ -8578,7 +8896,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H630"/>
+  <dimension ref="A1:H666"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -32107,6 +32425,1302 @@
       </c>
       <c r="H630" s="5" t="inlineStr"/>
     </row>
+    <row r="631">
+      <c r="A631" s="5" t="inlineStr">
+        <is>
+          <t>RDI-SPR-0008</t>
+        </is>
+      </c>
+      <c r="B631" s="5" t="inlineStr">
+        <is>
+          <t>source_area_name</t>
+        </is>
+      </c>
+      <c r="C631" s="5" t="inlineStr">
+        <is>
+          <t>Badeda village, Narendra Nagar block, Tehri Garhwal, Uttarakhand</t>
+        </is>
+      </c>
+      <c r="D631" s="5" t="inlineStr"/>
+      <c r="E631" s="5" t="inlineStr">
+        <is>
+          <t>descriptive</t>
+        </is>
+      </c>
+      <c r="F631" s="5" t="inlineStr">
+        <is>
+          <t>SRC-027</t>
+        </is>
+      </c>
+      <c r="G631" s="5" t="inlineStr">
+        <is>
+          <t>Badera Geohydrology  report.pdf, section 1 (Location and Site Characteristics)</t>
+        </is>
+      </c>
+      <c r="H631" s="5" t="inlineStr"/>
+    </row>
+    <row r="632">
+      <c r="A632" s="5" t="inlineStr">
+        <is>
+          <t>RDI-SPR-0008</t>
+        </is>
+      </c>
+      <c r="B632" s="5" t="inlineStr">
+        <is>
+          <t>district</t>
+        </is>
+      </c>
+      <c r="C632" s="5" t="inlineStr">
+        <is>
+          <t>Tehri Garhwal</t>
+        </is>
+      </c>
+      <c r="D632" s="5" t="inlineStr"/>
+      <c r="E632" s="5" t="inlineStr">
+        <is>
+          <t>descriptive</t>
+        </is>
+      </c>
+      <c r="F632" s="5" t="inlineStr">
+        <is>
+          <t>SRC-027</t>
+        </is>
+      </c>
+      <c r="G632" s="5" t="inlineStr">
+        <is>
+          <t>Badera Geohydrology  report.pdf, section 1 (Location and Site Characteristics)</t>
+        </is>
+      </c>
+      <c r="H632" s="5" t="inlineStr"/>
+    </row>
+    <row r="633">
+      <c r="A633" s="5" t="inlineStr">
+        <is>
+          <t>RDI-SPR-0008</t>
+        </is>
+      </c>
+      <c r="B633" s="5" t="inlineStr">
+        <is>
+          <t>block</t>
+        </is>
+      </c>
+      <c r="C633" s="5" t="inlineStr">
+        <is>
+          <t>Narendra Nagar</t>
+        </is>
+      </c>
+      <c r="D633" s="5" t="inlineStr"/>
+      <c r="E633" s="5" t="inlineStr">
+        <is>
+          <t>descriptive</t>
+        </is>
+      </c>
+      <c r="F633" s="5" t="inlineStr">
+        <is>
+          <t>SRC-027</t>
+        </is>
+      </c>
+      <c r="G633" s="5" t="inlineStr">
+        <is>
+          <t>Badera Geohydrology  report.pdf, section 1 (Location and Site Characteristics)</t>
+        </is>
+      </c>
+      <c r="H633" s="5" t="inlineStr"/>
+    </row>
+    <row r="634">
+      <c r="A634" s="5" t="inlineStr">
+        <is>
+          <t>RDI-SPR-0008</t>
+        </is>
+      </c>
+      <c r="B634" s="5" t="inlineStr">
+        <is>
+          <t>village</t>
+        </is>
+      </c>
+      <c r="C634" s="5" t="inlineStr">
+        <is>
+          <t>Badeda (Badera)</t>
+        </is>
+      </c>
+      <c r="D634" s="5" t="inlineStr"/>
+      <c r="E634" s="5" t="inlineStr">
+        <is>
+          <t>descriptive</t>
+        </is>
+      </c>
+      <c r="F634" s="5" t="inlineStr">
+        <is>
+          <t>SRC-027</t>
+        </is>
+      </c>
+      <c r="G634" s="5" t="inlineStr">
+        <is>
+          <t>Badera Geohydrology  report.pdf, section 1 (Location and Site Characteristics)</t>
+        </is>
+      </c>
+      <c r="H634" s="5" t="inlineStr"/>
+    </row>
+    <row r="635">
+      <c r="A635" s="5" t="inlineStr">
+        <is>
+          <t>RDI-SPR-0008</t>
+        </is>
+      </c>
+      <c r="B635" s="5" t="inlineStr">
+        <is>
+          <t>spring_name</t>
+        </is>
+      </c>
+      <c r="C635" s="5" t="inlineStr">
+        <is>
+          <t>Badeda Spring</t>
+        </is>
+      </c>
+      <c r="D635" s="5" t="inlineStr"/>
+      <c r="E635" s="5" t="inlineStr">
+        <is>
+          <t>descriptive</t>
+        </is>
+      </c>
+      <c r="F635" s="5" t="inlineStr">
+        <is>
+          <t>SRC-027</t>
+        </is>
+      </c>
+      <c r="G635" s="5" t="inlineStr">
+        <is>
+          <t>Badera Geohydrology  report.pdf, section 1 (Location and Site Characteristics)</t>
+        </is>
+      </c>
+      <c r="H635" s="5" t="inlineStr"/>
+    </row>
+    <row r="636">
+      <c r="A636" s="5" t="inlineStr">
+        <is>
+          <t>RDI-SPR-0008</t>
+        </is>
+      </c>
+      <c r="B636" s="5" t="inlineStr">
+        <is>
+          <t>latitude_source_value</t>
+        </is>
+      </c>
+      <c r="C636" s="5" t="inlineStr">
+        <is>
+          <t>30.171461</t>
+        </is>
+      </c>
+      <c r="D636" s="5" t="inlineStr">
+        <is>
+          <t>decimal degrees N</t>
+        </is>
+      </c>
+      <c r="E636" s="5" t="inlineStr">
+        <is>
+          <t>reported</t>
+        </is>
+      </c>
+      <c r="F636" s="5" t="inlineStr">
+        <is>
+          <t>SRC-027</t>
+        </is>
+      </c>
+      <c r="G636" s="5" t="inlineStr">
+        <is>
+          <t>Badera Geohydrology  report.pdf, section 1 (Location and Site Characteristics)</t>
+        </is>
+      </c>
+      <c r="H636" s="5" t="inlineStr">
+        <is>
+          <t>Printed as 30°10'17.26"N; converted to decimal degrees.</t>
+        </is>
+      </c>
+    </row>
+    <row r="637">
+      <c r="A637" s="5" t="inlineStr">
+        <is>
+          <t>RDI-SPR-0008</t>
+        </is>
+      </c>
+      <c r="B637" s="5" t="inlineStr">
+        <is>
+          <t>longitude_source_value</t>
+        </is>
+      </c>
+      <c r="C637" s="5" t="inlineStr">
+        <is>
+          <t>78.312894</t>
+        </is>
+      </c>
+      <c r="D637" s="5" t="inlineStr">
+        <is>
+          <t>decimal degrees E</t>
+        </is>
+      </c>
+      <c r="E637" s="5" t="inlineStr">
+        <is>
+          <t>reported</t>
+        </is>
+      </c>
+      <c r="F637" s="5" t="inlineStr">
+        <is>
+          <t>SRC-027</t>
+        </is>
+      </c>
+      <c r="G637" s="5" t="inlineStr">
+        <is>
+          <t>Badera Geohydrology  report.pdf, section 1 (Location and Site Characteristics)</t>
+        </is>
+      </c>
+      <c r="H637" s="5" t="inlineStr">
+        <is>
+          <t>Printed as 78°18'46.42"E; converted to decimal degrees.</t>
+        </is>
+      </c>
+    </row>
+    <row r="638">
+      <c r="A638" s="5" t="inlineStr">
+        <is>
+          <t>RDI-SPR-0008</t>
+        </is>
+      </c>
+      <c r="B638" s="5" t="inlineStr">
+        <is>
+          <t>land_use_source_value</t>
+        </is>
+      </c>
+      <c r="C638" s="5" t="inlineStr">
+        <is>
+          <t>Catchment: dense forest 48.4 %, open forest 16.0 %, agriculture/terrace 25.7 %, built-up 5.2 %, barren 3.2 %, road 1.5 % (Sentinel-2, 2025; the text says 66.91 % forest)</t>
+        </is>
+      </c>
+      <c r="D638" s="5" t="inlineStr"/>
+      <c r="E638" s="5" t="inlineStr">
+        <is>
+          <t>delineated_estimate</t>
+        </is>
+      </c>
+      <c r="F638" s="5" t="inlineStr">
+        <is>
+          <t>SRC-027</t>
+        </is>
+      </c>
+      <c r="G638" s="5" t="inlineStr">
+        <is>
+          <t>Badera Geohydrology  report.pdf, section 3.9</t>
+        </is>
+      </c>
+      <c r="H638" s="5" t="inlineStr"/>
+    </row>
+    <row r="639">
+      <c r="A639" s="5" t="inlineStr">
+        <is>
+          <t>RDI-SPR-0008</t>
+        </is>
+      </c>
+      <c r="B639" s="5" t="inlineStr">
+        <is>
+          <t>spring_type_source_value</t>
+        </is>
+      </c>
+      <c r="C639" s="5" t="inlineStr">
+        <is>
+          <t>Fracture-controlled contact spring; fractured to semi-confined carbonate aquifer of the Krol Group</t>
+        </is>
+      </c>
+      <c r="D639" s="5" t="inlineStr"/>
+      <c r="E639" s="5" t="inlineStr">
+        <is>
+          <t>descriptive</t>
+        </is>
+      </c>
+      <c r="F639" s="5" t="inlineStr">
+        <is>
+          <t>SRC-027</t>
+        </is>
+      </c>
+      <c r="G639" s="5" t="inlineStr">
+        <is>
+          <t>Badera Geohydrology  report.pdf, section 2</t>
+        </is>
+      </c>
+      <c r="H639" s="5" t="inlineStr"/>
+    </row>
+    <row r="640">
+      <c r="A640" s="5" t="inlineStr">
+        <is>
+          <t>RDI-SPR-0008</t>
+        </is>
+      </c>
+      <c r="B640" s="5" t="inlineStr">
+        <is>
+          <t>lithology_source_value</t>
+        </is>
+      </c>
+      <c r="C640" s="5" t="inlineStr">
+        <is>
+          <t>Limestone, dolomite and shale (Krol Group); aquifer table adds quartzite and sandstone (Blaini Group)</t>
+        </is>
+      </c>
+      <c r="D640" s="5" t="inlineStr"/>
+      <c r="E640" s="5" t="inlineStr">
+        <is>
+          <t>descriptive</t>
+        </is>
+      </c>
+      <c r="F640" s="5" t="inlineStr">
+        <is>
+          <t>SRC-027</t>
+        </is>
+      </c>
+      <c r="G640" s="5" t="inlineStr">
+        <is>
+          <t>Badera Geohydrology  report.pdf, sections 2, 3.6 and Table 1</t>
+        </is>
+      </c>
+      <c r="H640" s="5" t="inlineStr"/>
+    </row>
+    <row r="641">
+      <c r="A641" s="5" t="inlineStr">
+        <is>
+          <t>RDI-SPR-0008</t>
+        </is>
+      </c>
+      <c r="B641" s="5" t="inlineStr">
+        <is>
+          <t>geological_structure_source_value</t>
+        </is>
+      </c>
+      <c r="C641" s="5" t="inlineStr">
+        <is>
+          <t>Neoproterozoic Krol Group; groundwater controlled by fractures, joints and bedding planes; Highly Dissected Structural Hills and Valleys</t>
+        </is>
+      </c>
+      <c r="D641" s="5" t="inlineStr"/>
+      <c r="E641" s="5" t="inlineStr">
+        <is>
+          <t>descriptive</t>
+        </is>
+      </c>
+      <c r="F641" s="5" t="inlineStr">
+        <is>
+          <t>SRC-027</t>
+        </is>
+      </c>
+      <c r="G641" s="5" t="inlineStr">
+        <is>
+          <t>Badera Geohydrology  report.pdf, sections 3.6-3.7</t>
+        </is>
+      </c>
+      <c r="H641" s="5" t="inlineStr"/>
+    </row>
+    <row r="642">
+      <c r="A642" s="5" t="inlineStr">
+        <is>
+          <t>RDI-SPR-0008</t>
+        </is>
+      </c>
+      <c r="B642" s="5" t="inlineStr">
+        <is>
+          <t>porosity_source_value</t>
+        </is>
+      </c>
+      <c r="C642" s="5" t="inlineStr">
+        <is>
+          <t>Secondary porosity through fractures, joints and weathering (soil effective porosity 25-40 %)</t>
+        </is>
+      </c>
+      <c r="D642" s="5" t="inlineStr"/>
+      <c r="E642" s="5" t="inlineStr">
+        <is>
+          <t>descriptive</t>
+        </is>
+      </c>
+      <c r="F642" s="5" t="inlineStr">
+        <is>
+          <t>SRC-027</t>
+        </is>
+      </c>
+      <c r="G642" s="5" t="inlineStr">
+        <is>
+          <t>Badera Geohydrology  report.pdf, Table 1</t>
+        </is>
+      </c>
+      <c r="H642" s="5" t="inlineStr"/>
+    </row>
+    <row r="643">
+      <c r="A643" s="5" t="inlineStr">
+        <is>
+          <t>RDI-SPR-0008</t>
+        </is>
+      </c>
+      <c r="B643" s="5" t="inlineStr">
+        <is>
+          <t>seasonality_source_value</t>
+        </is>
+      </c>
+      <c r="C643" s="5" t="inlineStr">
+        <is>
+          <t>Perennial</t>
+        </is>
+      </c>
+      <c r="D643" s="5" t="inlineStr"/>
+      <c r="E643" s="5" t="inlineStr">
+        <is>
+          <t>reported</t>
+        </is>
+      </c>
+      <c r="F643" s="5" t="inlineStr">
+        <is>
+          <t>SRC-027</t>
+        </is>
+      </c>
+      <c r="G643" s="5" t="inlineStr">
+        <is>
+          <t>Badera Geohydrology  report.pdf, section 4</t>
+        </is>
+      </c>
+      <c r="H643" s="5" t="inlineStr">
+        <is>
+          <t>Section 4 lists 'presence of a perennial spring'.</t>
+        </is>
+      </c>
+    </row>
+    <row r="644">
+      <c r="A644" s="5" t="inlineStr">
+        <is>
+          <t>RDI-SPR-0008</t>
+        </is>
+      </c>
+      <c r="B644" s="5" t="inlineStr">
+        <is>
+          <t>catchment_area_ha_source_value</t>
+        </is>
+      </c>
+      <c r="C644" s="5" t="inlineStr">
+        <is>
+          <t>40.51</t>
+        </is>
+      </c>
+      <c r="D644" s="5" t="inlineStr">
+        <is>
+          <t>ha</t>
+        </is>
+      </c>
+      <c r="E644" s="5" t="inlineStr">
+        <is>
+          <t>delineated_estimate</t>
+        </is>
+      </c>
+      <c r="F644" s="5" t="inlineStr">
+        <is>
+          <t>SRC-027</t>
+        </is>
+      </c>
+      <c r="G644" s="5" t="inlineStr">
+        <is>
+          <t>Badera Geohydrology  report.pdf, Figure 10, Land Use / Land Cover Statistics table (total)</t>
+        </is>
+      </c>
+      <c r="H644" s="5" t="inlineStr">
+        <is>
+          <t>Surface catchment from CartoDEM 30 m; not a confirmed recharge area.</t>
+        </is>
+      </c>
+    </row>
+    <row r="645">
+      <c r="A645" s="5" t="inlineStr">
+        <is>
+          <t>RDI-SPR-0008</t>
+        </is>
+      </c>
+      <c r="B645" s="5" t="inlineStr">
+        <is>
+          <t>catchment_elevation_range_m_source_value</t>
+        </is>
+      </c>
+      <c r="C645" s="5" t="inlineStr">
+        <is>
+          <t>1452–1614</t>
+        </is>
+      </c>
+      <c r="D645" s="5" t="inlineStr">
+        <is>
+          <t>m asl</t>
+        </is>
+      </c>
+      <c r="E645" s="5" t="inlineStr">
+        <is>
+          <t>delineated_estimate</t>
+        </is>
+      </c>
+      <c r="F645" s="5" t="inlineStr">
+        <is>
+          <t>SRC-027</t>
+        </is>
+      </c>
+      <c r="G645" s="5" t="inlineStr">
+        <is>
+          <t>Badera Geohydrology  report.pdf, Section 3.1</t>
+        </is>
+      </c>
+      <c r="H645" s="5" t="inlineStr"/>
+    </row>
+    <row r="646">
+      <c r="A646" s="5" t="inlineStr">
+        <is>
+          <t>RDI-SPR-0008</t>
+        </is>
+      </c>
+      <c r="B646" s="5" t="inlineStr">
+        <is>
+          <t>recharge_area_slope_aspect_source_value</t>
+        </is>
+      </c>
+      <c r="C646" s="5" t="inlineStr">
+        <is>
+          <t>Slope 5–36° (12–28° around the handpump); mostly south- to southwest-facing</t>
+        </is>
+      </c>
+      <c r="D646" s="5" t="inlineStr"/>
+      <c r="E646" s="5" t="inlineStr">
+        <is>
+          <t>descriptive</t>
+        </is>
+      </c>
+      <c r="F646" s="5" t="inlineStr">
+        <is>
+          <t>SRC-027</t>
+        </is>
+      </c>
+      <c r="G646" s="5" t="inlineStr">
+        <is>
+          <t>Badera Geohydrology  report.pdf, sections 3.3-3.4</t>
+        </is>
+      </c>
+      <c r="H646" s="5" t="inlineStr"/>
+    </row>
+    <row r="647">
+      <c r="A647" s="5" t="inlineStr">
+        <is>
+          <t>RDI-SPR-0008</t>
+        </is>
+      </c>
+      <c r="B647" s="5" t="inlineStr">
+        <is>
+          <t>recharge_area_basis_source_value</t>
+        </is>
+      </c>
+      <c r="C647" s="5" t="inlineStr">
+        <is>
+          <t>Surface catchment from CartoDEM 30 m with thematic layers; the handpump area is called the upper recharge zone</t>
+        </is>
+      </c>
+      <c r="D647" s="5" t="inlineStr"/>
+      <c r="E647" s="5" t="inlineStr">
+        <is>
+          <t>descriptive</t>
+        </is>
+      </c>
+      <c r="F647" s="5" t="inlineStr">
+        <is>
+          <t>SRC-027</t>
+        </is>
+      </c>
+      <c r="G647" s="5" t="inlineStr">
+        <is>
+          <t>Badera Geohydrology  report.pdf, section 3</t>
+        </is>
+      </c>
+      <c r="H647" s="5" t="inlineStr"/>
+    </row>
+    <row r="648">
+      <c r="A648" s="5" t="inlineStr">
+        <is>
+          <t>RDI-SPR-0008</t>
+        </is>
+      </c>
+      <c r="B648" s="5" t="inlineStr">
+        <is>
+          <t>intervention_source_value</t>
+        </is>
+      </c>
+      <c r="C648" s="5" t="inlineStr">
+        <is>
+          <t>Rooftop rainwater harvesting with direct injection through the existing Badeda handpump (Kunjapuri; report: 'upper recharge zone of the Kunjapuri Spring catchment') at 30.173392, 78.312847, plus catchment treatment (trenches, recharge pits, check dams). The report places the handpump upslope of the spring in the same shallow fractured aquifer ('only a few metres apart'; the printed coordinates are about 215 m apart).</t>
+        </is>
+      </c>
+      <c r="D648" s="5" t="inlineStr"/>
+      <c r="E648" s="5" t="inlineStr">
+        <is>
+          <t>reported</t>
+        </is>
+      </c>
+      <c r="F648" s="5" t="inlineStr">
+        <is>
+          <t>SRC-027</t>
+        </is>
+      </c>
+      <c r="G648" s="5" t="inlineStr">
+        <is>
+          <t>Badera Geohydrology  report.pdf, sections 1-2 and 5</t>
+        </is>
+      </c>
+      <c r="H648" s="5" t="inlineStr">
+        <is>
+          <t>Handpump printed as 30°10'24.21"N 78°18'46.25"E.</t>
+        </is>
+      </c>
+    </row>
+    <row r="649">
+      <c r="A649" s="5" t="inlineStr">
+        <is>
+          <t>RDI-SPR-0009</t>
+        </is>
+      </c>
+      <c r="B649" s="5" t="inlineStr">
+        <is>
+          <t>source_area_name</t>
+        </is>
+      </c>
+      <c r="C649" s="5" t="inlineStr">
+        <is>
+          <t>Dungsi &amp; Makhdet villages, Jaunpur block, Tehri Garhwal, Uttarakhand</t>
+        </is>
+      </c>
+      <c r="D649" s="5" t="inlineStr"/>
+      <c r="E649" s="5" t="inlineStr">
+        <is>
+          <t>descriptive</t>
+        </is>
+      </c>
+      <c r="F649" s="5" t="inlineStr">
+        <is>
+          <t>SRC-028</t>
+        </is>
+      </c>
+      <c r="G649" s="5" t="inlineStr">
+        <is>
+          <t>Domsi &amp; Makhdet Geohydrology report.pdf, section 1 (Location and Site Characteristics)</t>
+        </is>
+      </c>
+      <c r="H649" s="5" t="inlineStr"/>
+    </row>
+    <row r="650">
+      <c r="A650" s="5" t="inlineStr">
+        <is>
+          <t>RDI-SPR-0009</t>
+        </is>
+      </c>
+      <c r="B650" s="5" t="inlineStr">
+        <is>
+          <t>district</t>
+        </is>
+      </c>
+      <c r="C650" s="5" t="inlineStr">
+        <is>
+          <t>Tehri Garhwal</t>
+        </is>
+      </c>
+      <c r="D650" s="5" t="inlineStr"/>
+      <c r="E650" s="5" t="inlineStr">
+        <is>
+          <t>descriptive</t>
+        </is>
+      </c>
+      <c r="F650" s="5" t="inlineStr">
+        <is>
+          <t>SRC-028</t>
+        </is>
+      </c>
+      <c r="G650" s="5" t="inlineStr">
+        <is>
+          <t>Domsi &amp; Makhdet Geohydrology report.pdf, section 1 (Location and Site Characteristics)</t>
+        </is>
+      </c>
+      <c r="H650" s="5" t="inlineStr"/>
+    </row>
+    <row r="651">
+      <c r="A651" s="5" t="inlineStr">
+        <is>
+          <t>RDI-SPR-0009</t>
+        </is>
+      </c>
+      <c r="B651" s="5" t="inlineStr">
+        <is>
+          <t>block</t>
+        </is>
+      </c>
+      <c r="C651" s="5" t="inlineStr">
+        <is>
+          <t>Jaunpur</t>
+        </is>
+      </c>
+      <c r="D651" s="5" t="inlineStr"/>
+      <c r="E651" s="5" t="inlineStr">
+        <is>
+          <t>descriptive</t>
+        </is>
+      </c>
+      <c r="F651" s="5" t="inlineStr">
+        <is>
+          <t>SRC-028</t>
+        </is>
+      </c>
+      <c r="G651" s="5" t="inlineStr">
+        <is>
+          <t>Domsi &amp; Makhdet Geohydrology report.pdf, section 1 (Location and Site Characteristics)</t>
+        </is>
+      </c>
+      <c r="H651" s="5" t="inlineStr"/>
+    </row>
+    <row r="652">
+      <c r="A652" s="5" t="inlineStr">
+        <is>
+          <t>RDI-SPR-0009</t>
+        </is>
+      </c>
+      <c r="B652" s="5" t="inlineStr">
+        <is>
+          <t>village</t>
+        </is>
+      </c>
+      <c r="C652" s="5" t="inlineStr">
+        <is>
+          <t>Makhdet (Dungsi &amp; Makhdet; also spelt Madkhet, Domsi)</t>
+        </is>
+      </c>
+      <c r="D652" s="5" t="inlineStr"/>
+      <c r="E652" s="5" t="inlineStr">
+        <is>
+          <t>descriptive</t>
+        </is>
+      </c>
+      <c r="F652" s="5" t="inlineStr">
+        <is>
+          <t>SRC-028</t>
+        </is>
+      </c>
+      <c r="G652" s="5" t="inlineStr">
+        <is>
+          <t>Domsi &amp; Makhdet Geohydrology report.pdf, section 1 (Location and Site Characteristics)</t>
+        </is>
+      </c>
+      <c r="H652" s="5" t="inlineStr"/>
+    </row>
+    <row r="653">
+      <c r="A653" s="5" t="inlineStr">
+        <is>
+          <t>RDI-SPR-0009</t>
+        </is>
+      </c>
+      <c r="B653" s="5" t="inlineStr">
+        <is>
+          <t>spring_name</t>
+        </is>
+      </c>
+      <c r="C653" s="5" t="inlineStr">
+        <is>
+          <t>Makhdet Spring</t>
+        </is>
+      </c>
+      <c r="D653" s="5" t="inlineStr"/>
+      <c r="E653" s="5" t="inlineStr">
+        <is>
+          <t>descriptive</t>
+        </is>
+      </c>
+      <c r="F653" s="5" t="inlineStr">
+        <is>
+          <t>SRC-028</t>
+        </is>
+      </c>
+      <c r="G653" s="5" t="inlineStr">
+        <is>
+          <t>Domsi &amp; Makhdet Geohydrology report.pdf, section 1 (Location and Site Characteristics)</t>
+        </is>
+      </c>
+      <c r="H653" s="5" t="inlineStr"/>
+    </row>
+    <row r="654">
+      <c r="A654" s="5" t="inlineStr">
+        <is>
+          <t>RDI-SPR-0009</t>
+        </is>
+      </c>
+      <c r="B654" s="5" t="inlineStr">
+        <is>
+          <t>latitude_source_value</t>
+        </is>
+      </c>
+      <c r="C654" s="5" t="inlineStr">
+        <is>
+          <t>30.482739</t>
+        </is>
+      </c>
+      <c r="D654" s="5" t="inlineStr">
+        <is>
+          <t>decimal degrees N</t>
+        </is>
+      </c>
+      <c r="E654" s="5" t="inlineStr">
+        <is>
+          <t>reported</t>
+        </is>
+      </c>
+      <c r="F654" s="5" t="inlineStr">
+        <is>
+          <t>SRC-028</t>
+        </is>
+      </c>
+      <c r="G654" s="5" t="inlineStr">
+        <is>
+          <t>Domsi &amp; Makhdet Geohydrology report.pdf, section 1 (Location and Site Characteristics)</t>
+        </is>
+      </c>
+      <c r="H654" s="5" t="inlineStr">
+        <is>
+          <t>Printed as 30°28'57.86"N; converted to decimal degrees.</t>
+        </is>
+      </c>
+    </row>
+    <row r="655">
+      <c r="A655" s="5" t="inlineStr">
+        <is>
+          <t>RDI-SPR-0009</t>
+        </is>
+      </c>
+      <c r="B655" s="5" t="inlineStr">
+        <is>
+          <t>longitude_source_value</t>
+        </is>
+      </c>
+      <c r="C655" s="5" t="inlineStr">
+        <is>
+          <t>78.234675</t>
+        </is>
+      </c>
+      <c r="D655" s="5" t="inlineStr">
+        <is>
+          <t>decimal degrees E</t>
+        </is>
+      </c>
+      <c r="E655" s="5" t="inlineStr">
+        <is>
+          <t>reported</t>
+        </is>
+      </c>
+      <c r="F655" s="5" t="inlineStr">
+        <is>
+          <t>SRC-028</t>
+        </is>
+      </c>
+      <c r="G655" s="5" t="inlineStr">
+        <is>
+          <t>Domsi &amp; Makhdet Geohydrology report.pdf, section 1 (Location and Site Characteristics)</t>
+        </is>
+      </c>
+      <c r="H655" s="5" t="inlineStr">
+        <is>
+          <t>Printed as 78°14'4.83"E; converted to decimal degrees.</t>
+        </is>
+      </c>
+    </row>
+    <row r="656">
+      <c r="A656" s="5" t="inlineStr">
+        <is>
+          <t>RDI-SPR-0009</t>
+        </is>
+      </c>
+      <c r="B656" s="5" t="inlineStr">
+        <is>
+          <t>land_use_source_value</t>
+        </is>
+      </c>
+      <c r="C656" s="5" t="inlineStr">
+        <is>
+          <t>Catchment: dense forest 40.8 %, open forest 25.4 %, agriculture/terrace 22.6 %, built-up 4.3 %, barren 3.5 %, road 1.3 %, water 0.3 % (Sentinel-2, 2025)</t>
+        </is>
+      </c>
+      <c r="D656" s="5" t="inlineStr"/>
+      <c r="E656" s="5" t="inlineStr">
+        <is>
+          <t>delineated_estimate</t>
+        </is>
+      </c>
+      <c r="F656" s="5" t="inlineStr">
+        <is>
+          <t>SRC-028</t>
+        </is>
+      </c>
+      <c r="G656" s="5" t="inlineStr">
+        <is>
+          <t>Domsi &amp; Makhdet Geohydrology report.pdf, section 3.9</t>
+        </is>
+      </c>
+      <c r="H656" s="5" t="inlineStr"/>
+    </row>
+    <row r="657">
+      <c r="A657" s="5" t="inlineStr">
+        <is>
+          <t>RDI-SPR-0009</t>
+        </is>
+      </c>
+      <c r="B657" s="5" t="inlineStr">
+        <is>
+          <t>spring_type_source_value</t>
+        </is>
+      </c>
+      <c r="C657" s="5" t="inlineStr">
+        <is>
+          <t>Fracture-controlled gravity spring; unconfined to semi-confined fractured hard-rock aquifer</t>
+        </is>
+      </c>
+      <c r="D657" s="5" t="inlineStr"/>
+      <c r="E657" s="5" t="inlineStr">
+        <is>
+          <t>descriptive</t>
+        </is>
+      </c>
+      <c r="F657" s="5" t="inlineStr">
+        <is>
+          <t>SRC-028</t>
+        </is>
+      </c>
+      <c r="G657" s="5" t="inlineStr">
+        <is>
+          <t>Domsi &amp; Makhdet Geohydrology report.pdf, section 2</t>
+        </is>
+      </c>
+      <c r="H657" s="5" t="inlineStr"/>
+    </row>
+    <row r="658">
+      <c r="A658" s="5" t="inlineStr">
+        <is>
+          <t>RDI-SPR-0009</t>
+        </is>
+      </c>
+      <c r="B658" s="5" t="inlineStr">
+        <is>
+          <t>lithology_source_value</t>
+        </is>
+      </c>
+      <c r="C658" s="5" t="inlineStr">
+        <is>
+          <t>Quartzite, phyllite, slate and schist (Jaunsar Group; the aquifer table says Jaunpur Group)</t>
+        </is>
+      </c>
+      <c r="D658" s="5" t="inlineStr"/>
+      <c r="E658" s="5" t="inlineStr">
+        <is>
+          <t>descriptive</t>
+        </is>
+      </c>
+      <c r="F658" s="5" t="inlineStr">
+        <is>
+          <t>SRC-028</t>
+        </is>
+      </c>
+      <c r="G658" s="5" t="inlineStr">
+        <is>
+          <t>Domsi &amp; Makhdet Geohydrology report.pdf, sections 2, 3.6 and Table 1</t>
+        </is>
+      </c>
+      <c r="H658" s="5" t="inlineStr"/>
+    </row>
+    <row r="659">
+      <c r="A659" s="5" t="inlineStr">
+        <is>
+          <t>RDI-SPR-0009</t>
+        </is>
+      </c>
+      <c r="B659" s="5" t="inlineStr">
+        <is>
+          <t>geological_structure_source_value</t>
+        </is>
+      </c>
+      <c r="C659" s="5" t="inlineStr">
+        <is>
+          <t>Neoproterozoic Jaunsar Group, Lesser Himalaya; groundwater controlled by fractures, joints, foliation and bedding planes; Highly Dissected Hills and Valleys</t>
+        </is>
+      </c>
+      <c r="D659" s="5" t="inlineStr"/>
+      <c r="E659" s="5" t="inlineStr">
+        <is>
+          <t>descriptive</t>
+        </is>
+      </c>
+      <c r="F659" s="5" t="inlineStr">
+        <is>
+          <t>SRC-028</t>
+        </is>
+      </c>
+      <c r="G659" s="5" t="inlineStr">
+        <is>
+          <t>Domsi &amp; Makhdet Geohydrology report.pdf, sections 3.6-3.7</t>
+        </is>
+      </c>
+      <c r="H659" s="5" t="inlineStr"/>
+    </row>
+    <row r="660">
+      <c r="A660" s="5" t="inlineStr">
+        <is>
+          <t>RDI-SPR-0009</t>
+        </is>
+      </c>
+      <c r="B660" s="5" t="inlineStr">
+        <is>
+          <t>porosity_source_value</t>
+        </is>
+      </c>
+      <c r="C660" s="5" t="inlineStr">
+        <is>
+          <t>Secondary porosity through fractures, joints, foliation and weathering (soil effective porosity 20-35 %)</t>
+        </is>
+      </c>
+      <c r="D660" s="5" t="inlineStr"/>
+      <c r="E660" s="5" t="inlineStr">
+        <is>
+          <t>descriptive</t>
+        </is>
+      </c>
+      <c r="F660" s="5" t="inlineStr">
+        <is>
+          <t>SRC-028</t>
+        </is>
+      </c>
+      <c r="G660" s="5" t="inlineStr">
+        <is>
+          <t>Domsi &amp; Makhdet Geohydrology report.pdf, Table 1</t>
+        </is>
+      </c>
+      <c r="H660" s="5" t="inlineStr"/>
+    </row>
+    <row r="661">
+      <c r="A661" s="5" t="inlineStr">
+        <is>
+          <t>RDI-SPR-0009</t>
+        </is>
+      </c>
+      <c r="B661" s="5" t="inlineStr">
+        <is>
+          <t>seasonality_source_value</t>
+        </is>
+      </c>
+      <c r="C661" s="5" t="inlineStr">
+        <is>
+          <t>Perennial</t>
+        </is>
+      </c>
+      <c r="D661" s="5" t="inlineStr"/>
+      <c r="E661" s="5" t="inlineStr">
+        <is>
+          <t>reported</t>
+        </is>
+      </c>
+      <c r="F661" s="5" t="inlineStr">
+        <is>
+          <t>SRC-028</t>
+        </is>
+      </c>
+      <c r="G661" s="5" t="inlineStr">
+        <is>
+          <t>Domsi &amp; Makhdet Geohydrology report.pdf, section 4</t>
+        </is>
+      </c>
+      <c r="H661" s="5" t="inlineStr">
+        <is>
+          <t>Section 4 lists 'presence of a perennial spring'.</t>
+        </is>
+      </c>
+    </row>
+    <row r="662">
+      <c r="A662" s="5" t="inlineStr">
+        <is>
+          <t>RDI-SPR-0009</t>
+        </is>
+      </c>
+      <c r="B662" s="5" t="inlineStr">
+        <is>
+          <t>catchment_area_ha_source_value</t>
+        </is>
+      </c>
+      <c r="C662" s="5" t="inlineStr">
+        <is>
+          <t>91.07</t>
+        </is>
+      </c>
+      <c r="D662" s="5" t="inlineStr">
+        <is>
+          <t>ha</t>
+        </is>
+      </c>
+      <c r="E662" s="5" t="inlineStr">
+        <is>
+          <t>delineated_estimate</t>
+        </is>
+      </c>
+      <c r="F662" s="5" t="inlineStr">
+        <is>
+          <t>SRC-028</t>
+        </is>
+      </c>
+      <c r="G662" s="5" t="inlineStr">
+        <is>
+          <t>Domsi &amp; Makhdet Geohydrology report.pdf, Section 3.9 (delineated catchment)</t>
+        </is>
+      </c>
+      <c r="H662" s="5" t="inlineStr">
+        <is>
+          <t>Surface catchment from CartoDEM 30 m; not a confirmed recharge area.</t>
+        </is>
+      </c>
+    </row>
+    <row r="663">
+      <c r="A663" s="5" t="inlineStr">
+        <is>
+          <t>RDI-SPR-0009</t>
+        </is>
+      </c>
+      <c r="B663" s="5" t="inlineStr">
+        <is>
+          <t>catchment_elevation_range_m_source_value</t>
+        </is>
+      </c>
+      <c r="C663" s="5" t="inlineStr">
+        <is>
+          <t>1461–2076</t>
+        </is>
+      </c>
+      <c r="D663" s="5" t="inlineStr">
+        <is>
+          <t>m asl</t>
+        </is>
+      </c>
+      <c r="E663" s="5" t="inlineStr">
+        <is>
+          <t>delineated_estimate</t>
+        </is>
+      </c>
+      <c r="F663" s="5" t="inlineStr">
+        <is>
+          <t>SRC-028</t>
+        </is>
+      </c>
+      <c r="G663" s="5" t="inlineStr">
+        <is>
+          <t>Domsi &amp; Makhdet Geohydrology report.pdf, Sections 3.1 and 6.7 (section 3.5 gives about 1500–2050 from contours)</t>
+        </is>
+      </c>
+      <c r="H663" s="5" t="inlineStr"/>
+    </row>
+    <row r="664">
+      <c r="A664" s="5" t="inlineStr">
+        <is>
+          <t>RDI-SPR-0009</t>
+        </is>
+      </c>
+      <c r="B664" s="5" t="inlineStr">
+        <is>
+          <t>recharge_area_slope_aspect_source_value</t>
+        </is>
+      </c>
+      <c r="C664" s="5" t="inlineStr">
+        <is>
+          <t>Slope 5 to over 37° (5–15° around the spring and handpump); spring and handpump on northwest-facing slopes</t>
+        </is>
+      </c>
+      <c r="D664" s="5" t="inlineStr"/>
+      <c r="E664" s="5" t="inlineStr">
+        <is>
+          <t>descriptive</t>
+        </is>
+      </c>
+      <c r="F664" s="5" t="inlineStr">
+        <is>
+          <t>SRC-028</t>
+        </is>
+      </c>
+      <c r="G664" s="5" t="inlineStr">
+        <is>
+          <t>Domsi &amp; Makhdet Geohydrology report.pdf, sections 3.3-3.4</t>
+        </is>
+      </c>
+      <c r="H664" s="5" t="inlineStr"/>
+    </row>
+    <row r="665">
+      <c r="A665" s="5" t="inlineStr">
+        <is>
+          <t>RDI-SPR-0009</t>
+        </is>
+      </c>
+      <c r="B665" s="5" t="inlineStr">
+        <is>
+          <t>recharge_area_basis_source_value</t>
+        </is>
+      </c>
+      <c r="C665" s="5" t="inlineStr">
+        <is>
+          <t>Surface catchment from CartoDEM 30 m with thematic layers; the handpump area is called the upper recharge zone</t>
+        </is>
+      </c>
+      <c r="D665" s="5" t="inlineStr"/>
+      <c r="E665" s="5" t="inlineStr">
+        <is>
+          <t>descriptive</t>
+        </is>
+      </c>
+      <c r="F665" s="5" t="inlineStr">
+        <is>
+          <t>SRC-028</t>
+        </is>
+      </c>
+      <c r="G665" s="5" t="inlineStr">
+        <is>
+          <t>Domsi &amp; Makhdet Geohydrology report.pdf, section 3</t>
+        </is>
+      </c>
+      <c r="H665" s="5" t="inlineStr"/>
+    </row>
+    <row r="666">
+      <c r="A666" s="5" t="inlineStr">
+        <is>
+          <t>RDI-SPR-0009</t>
+        </is>
+      </c>
+      <c r="B666" s="5" t="inlineStr">
+        <is>
+          <t>intervention_source_value</t>
+        </is>
+      </c>
+      <c r="C666" s="5" t="inlineStr">
+        <is>
+          <t>Rooftop rainwater harvesting with direct injection through the existing Dungsi (Domsi) handpump at 30.481472, 78.236694, plus catchment treatment (trenches, recharge pits, check dams). The report places the handpump upslope of the spring in the same springshed, with 'probable hydraulic connectivity' through the fractured aquifer.</t>
+        </is>
+      </c>
+      <c r="D666" s="5" t="inlineStr"/>
+      <c r="E666" s="5" t="inlineStr">
+        <is>
+          <t>reported</t>
+        </is>
+      </c>
+      <c r="F666" s="5" t="inlineStr">
+        <is>
+          <t>SRC-028</t>
+        </is>
+      </c>
+      <c r="G666" s="5" t="inlineStr">
+        <is>
+          <t>Domsi &amp; Makhdet Geohydrology report.pdf, sections 1-2 and 5</t>
+        </is>
+      </c>
+      <c r="H666" s="5" t="inlineStr">
+        <is>
+          <t>Handpump printed as 30°28'53.3"N 78°14'12.1"E.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Record the new secondary data layers and trace the report catchments
Data only; no model changes (Rajat, 2026-10-22).
- Source register SRC-029 to SRC-033: Bhukosh 250k geomorphology, lineaments,
  landslide polygons, 50K oriented structure planes (Kumaon only), Sentinel-2.
- Transformation log TRN-017 to TRN-019; TRN-016 quoting fixed.
- Acquisition queue AQ-013 to AQ-015: soil depth, Tehri dip, NRSC 1:50k.
- scripts/build_sentinel2_ndvi.py, build_soil_infiltration.py,
  trace_report_catchments.py and the traced Badeda/Makhdet catchments.
- Badeda's 40.51 ha flagged: its own outline measures 12.4 ha.
- docs/secondary-data-inventory.md lists every layer and its status.

Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01SYEMBaPiJtYrK4Gc2Fn2t3
</commit_message>
<xml_diff>
--- a/data/01_staged/literature/xlsx/literature_spring_records_common_v1.xlsx
+++ b/data/01_staged/literature/xlsx/literature_spring_records_common_v1.xlsx
@@ -32925,7 +32925,7 @@
       </c>
       <c r="H644" s="5" t="inlineStr">
         <is>
-          <t>Surface catchment from CartoDEM 30 m; not a confirmed recharge area.</t>
+          <t>Surface catchment from CartoDEM 30 m; not a confirmed recharge area. The outline drawn on the report's other maps measures 12.4 ha (scripts/trace_report_catchments.py); the land-use map that gives 40.51 ha looks redrawn (repeated grid labels, UTM 43N), so prefer 12.4 ha.</t>
         </is>
       </c>
     </row>
@@ -33573,7 +33573,7 @@
       </c>
       <c r="H662" s="5" t="inlineStr">
         <is>
-          <t>Surface catchment from CartoDEM 30 m; not a confirmed recharge area.</t>
+          <t>Surface catchment from CartoDEM 30 m; not a confirmed recharge area. The outline on the report's geology map measures 94.3 ha (scripts/trace_report_catchments.py).</t>
         </is>
       </c>
     </row>

</xml_diff>